<commit_message>
docs(hub): FW-16 Done; FW-10 + FW-24 Dropped (owner 2026-07-05)
FW-16 Voice Dispatcher prod write verified working. FW-10 in-app reschedule and
FW-24 onboarding serviceStates killed by owner (covered elsewhere / redundant).
IDs retained per the numbering rule. Now 7 Done / 7 Partial / 2 Dropped / 35 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,11 +47,15 @@
       <color rgb="009C6500"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="001E7A34"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -148,6 +157,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -531,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - verified vs code 2026-07-05  |  6 Done, 10 Partial, 35 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  7 Done, 7 Partial, 2 Dropped, 35 Open</t>
         </is>
       </c>
     </row>
@@ -946,14 +958,14 @@
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Desktop drag-to-move across days + voice move work; no date/time reschedule picker on the job popup.</t>
+          <t>KILLED by owner 2026-07-05 — not pursuing (desktop drag-move + voice move already cover this).</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1148,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1174,14 +1186,14 @@
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr"/>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Write path fully wired (execute-&gt;method16 move/cancel/duration) but NOT prod-write-verified (dev VONIGO_READONLY); unified popup not mirrored on Manage Jobs voice bar.</t>
+          <t>VERIFIED DONE — owner confirms the dispatcher write path (move/cancel/duration) works in prod, 2026-07-05.</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1376,7 @@
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1478,14 +1490,14 @@
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>serviceStates captured/editable + feeds Town Price Lookup; per-estimator default state parked + signup-time capture not started.</t>
+          <t>KILLED by owner 2026-07-05 — native users already enter ZIPs in pricing; redundant.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1756,7 @@
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="11" t="inlineStr">
+      <c r="G33" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1820,7 +1832,7 @@
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="11" t="inlineStr">
+      <c r="G35" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1972,7 +1984,7 @@
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="11" t="inlineStr">
+      <c r="G39" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -2010,7 +2022,7 @@
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr"/>
-      <c r="G40" s="11" t="inlineStr">
+      <c r="G40" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
docs(hub): FW-51 Done (confirm-email inbox delivery tested, owner 2026-07-05)
Now 8 Done / 6 Partial / 2 Dropped / 35 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -543,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  7 Done, 7 Partial, 2 Dropped, 35 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  8 Done, 6 Partial, 2 Dropped, 35 Open</t>
         </is>
       </c>
     </row>
@@ -2516,14 +2516,14 @@
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>DMARC/SPF/DKIM done; real-signup inbox re-test remains (runtime).</t>
+          <t>VERIFIED DONE — owner tested confirm-email inbox delivery, working 2026-07-05 (DMARC/SPF/DKIM).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(hub): FW-46 Done — keys never left the machine, no rotation needed (owner 2026-07-05)
Now 9 Done / 5 Partial / 2 Dropped / 35 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -543,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  8 Done, 6 Partial, 2 Dropped, 35 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  9 Done, 5 Partial, 2 Dropped, 35 Open</t>
         </is>
       </c>
     </row>
@@ -2326,14 +2326,14 @@
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr"/>
-      <c r="G48" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>Local n8n export REDACTED to MY_* placeholders (Google/Anthropic/Motive keys + Sheet ID) + backup with real keys DELETED 2026-07-05; verified not in repo/history/index. Remaining: rotate ONLY if the original ever synced to cloud/shared (else close).</t>
+          <t>VERIFIED DONE 2026-07-05 — export redacted to MY_* placeholders + real-key backup deleted; verified not in repo/history/index; owner confirms the file never synced/shared → keys never left the machine, no rotation needed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(hub): FW-03 Done — #90 Motive already live in prod (verified 2026-07-05)
Verified prod #90: pull token connected (3 trucks) + webhook secret configured;
migration 0033 preserved it, so the re-entry FW-03 assumed was never needed.
Now 10 Done / 5 Partial / 2 Dropped / 34 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -44,15 +44,15 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001E7A34"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="009C6500"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="00808080"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001E7A34"/>
     </font>
   </fonts>
   <fills count="9">
@@ -84,17 +84,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -543,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  9 Done, 5 Partial, 2 Dropped, 35 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  10 Done, 5 Partial, 2 Dropped, 34 Open</t>
         </is>
       </c>
     </row>
@@ -692,14 +692,14 @@
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Owner action — per-franchise Vault token doesn't carry dev-&gt;prod; re-enter #90 Motive token in prod Settings.</t>
+          <t>VERIFIED DONE 2026-07-05 — prod #90 Motive already set up: pull token connected (3 trucks, telematics_credentials is_active) + webhook secret configured (motive_webhook_config). Migration 0033 preserved it; re-entry was never actually needed. (Prod validation stamp June 12; re-save on app.crewlogicai.com to refresh — optional.)</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr"/>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="11" t="inlineStr">
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr"/>
-      <c r="G28" s="10" t="inlineStr">
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="G33" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="12" t="inlineStr">
+      <c r="G35" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr"/>
-      <c r="G36" s="10" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -1984,7 +1984,7 @@
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="12" t="inlineStr">
+      <c r="G39" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -2022,7 +2022,7 @@
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr"/>
-      <c r="G40" s="12" t="inlineStr">
+      <c r="G40" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="10" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr"/>
-      <c r="G48" s="12" t="inlineStr">
+      <c r="G48" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="12" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
docs(hub): FW-14 Dropped (owner 2026-07-05); FW-17 confirmed still open
FW-14 weather narrow-scope killed. FW-17 town title-case verified NOT done
(townFromAddress returns raw uppercase; display doesn't title-case) — left Open
pending owner decision. Now 10 Done / 5 Partial / 3 Dropped / 33 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -543,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  10 Done, 5 Partial, 2 Dropped, 34 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  10 Done, 5 Partial, 3 Dropped, 33 Open</t>
         </is>
       </c>
     </row>
@@ -1110,14 +1110,14 @@
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>crewlogic-weather is state-level; dashboard + Job Plan only; not narrowed to office point, not on trucks screen.</t>
+          <t>KILLED by owner 2026-07-05 — not needed (state-level weather on dashboard + Job Plan is sufficient).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(hub): FW-17 + FW-22 Done — shipped to prod v5.50.2 (2026-07-05)
Now 12 Done / 5 Partial / 3 Dropped / 31 Open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CrewLogic-Future-Work-Register.xlsx
+++ b/docs/CrewLogic-Future-Work-Register.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,12 +54,8 @@
       <i val="1"/>
       <color rgb="00808080"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -101,11 +97,6 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -169,9 +160,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,7 +543,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  10 Done, 2 In progress, 5 Partial, 3 Dropped, 31 Open</t>
+          <t>CrewLogic Future-Work Register - stable IDs FW-01..FW-51 (do NOT renumber) - 2026-07-05  |  12 Done, 5 Partial, 3 Dropped, 31 Open</t>
         </is>
       </c>
     </row>
@@ -1236,14 +1224,14 @@
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>BUILT ON DEV v5.50.2 — town/city title-cased on job ALERTS (_geofenceAlertRow) AND the schedule board (job chip + hover/sticky popup City row) via _titleCaseTown. Other surfaces (price-lookup town list, customer list) left as-is unless flagged. Pending owner test + prod approval.</t>
+          <t>VERIFIED DONE (prod v5.50.2, 2026-07-05) — town/city title-cased on job ALERTS (_geofenceAlertRow) AND the schedule board (job chip + hover/sticky popup City row) via _titleCaseTown. Client names untouched. Other surfaces (price-lookup, customer list) intentionally left as-is.</t>
         </is>
       </c>
     </row>
@@ -1426,14 +1414,14 @@
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr"/>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>BUILT ON DEV v5.50.1 — calcShed rewritten: walls + floor + PITCHED roof debris volume with floor-joist / roof-rafter / shingle-layer inputs + on-screen component breakdown (~1.55x the old structure figure; fixes the missing-roof undercount). Pending owner test/calibration + prod approval.</t>
+          <t>VERIFIED DONE (prod v5.50.2, 2026-07-05) — calcShed rewritten: walls + floor + PITCHED roof debris volume with floor-joist / roof-rafter / shingle-layer inputs + on-screen walls/floor/roof breakdown (fixes the missing-roof undercount). Owner-tested/approved. Thickness factors remain calibratable if field use shows drift.</t>
         </is>
       </c>
     </row>

</xml_diff>